<commit_message>
feat: versão estável OptiGen V3 (engine + melhorias)
</commit_message>
<xml_diff>
--- a/data/DadosSedimentation.xlsx
+++ b/data/DadosSedimentation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Izaq\PycharmProjects\PythonProject\NewGen_DataLayer_FullProject\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Izaq\Projects\optigen-backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{556CCB0D-D3AE-4649-8B29-32BAA1A32BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC9C2A18-2F22-4BBA-B628-FCC6B2FF1D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{7C89A78E-0117-400B-BF16-4A00B9D07968}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{7C89A78E-0117-400B-BF16-4A00B9D07968}"/>
   </bookViews>
   <sheets>
     <sheet name="fluids_meta" sheetId="2" r:id="rId1"/>
@@ -3464,17 +3464,18 @@
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A190" s="14">
-        <v>5</v>
-      </c>
-      <c r="B190" s="3">
+      <c r="A190" s="10">
+        <v>5</v>
+      </c>
+      <c r="B190" s="6">
         <v>16</v>
       </c>
-      <c r="C190" s="3">
+      <c r="C190" s="6">
         <v>12</v>
       </c>
-      <c r="D190" s="3">
-        <v>6.6503770030326523E-2</v>
+      <c r="D190" s="6">
+        <f>AVERAGE(D189,D191)</f>
+        <v>2.7951989346897563E-2</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.3">
@@ -3968,17 +3969,18 @@
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A226" s="14">
-        <v>5</v>
-      </c>
-      <c r="B226" s="3">
+      <c r="A226" s="10">
+        <v>5</v>
+      </c>
+      <c r="B226" s="6">
         <v>18</v>
       </c>
-      <c r="C226" s="3">
+      <c r="C226" s="6">
         <v>12</v>
       </c>
-      <c r="D226" s="3">
-        <v>2.469552797563121E-2</v>
+      <c r="D226" s="6">
+        <f>AVERAGE(D225,D227)</f>
+        <v>7.8787870411198488E-3</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>